<commit_message>
State pages for the week ending 2026-10-25 (published from the PanelReady PC)
</commit_message>
<xml_diff>
--- a/sample/panelready-sample.xlsx
+++ b/sample/panelready-sample.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'New practices'!$A$4:$V$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'New practices'!$A$4:$Z$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'New practices'!$A$1:$O$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'New practices'!$4:$4</definedName>
   </definedNames>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="260">
   <si>
     <t>PanelReady</t>
   </si>
@@ -32,19 +32,19 @@
     <t>PANELREADY · SAMPLE LIST</t>
   </si>
   <si>
-    <t>Delaware</t>
-  </si>
-  <si>
-    <t>New healthcare practices, week ending October 18, 2026</t>
-  </si>
-  <si>
-    <t>October 23, 2026</t>
+    <t>Vermont</t>
+  </si>
+  <si>
+    <t>New healthcare practices, week ending October 25, 2026</t>
+  </si>
+  <si>
+    <t>October 26, 2026</t>
   </si>
   <si>
     <t>New practices  ›</t>
   </si>
   <si>
-    <t>This sample is every new practice that registered in Delaware in the week ending October 18, 2026, scored and sorted the way subscribers get their own state, every week. Subscribers' lists also have the websites and emails we find for organizations, the practices that moved or added a specialty, and an OIG exclusion check.</t>
+    <t>This sample is every new practice that registered in Vermont in the week ending October 25, 2026, scored and sorted the way subscribers get their own state, every week. Subscribers' lists also have the websites and emails we find for organizations, the practices that moved or added a specialty, and an OIG exclusion check.</t>
   </si>
   <si>
     <t>Hottest leads</t>
@@ -65,118 +65,112 @@
     <t>NPI</t>
   </si>
   <si>
-    <t>Infusion Center of Delaware</t>
-  </si>
-  <si>
-    <t>Internal Medicine, Rheumatology</t>
-  </si>
-  <si>
-    <t>Dover, DE</t>
-  </si>
-  <si>
-    <t>1942106075</t>
-  </si>
-  <si>
-    <t>Allminds Medical Group Midwest PA</t>
-  </si>
-  <si>
-    <t>Clinic/Center, Mental Health (Including Community Mental Health Center)</t>
-  </si>
-  <si>
-    <t>Wilmington, DE</t>
-  </si>
-  <si>
-    <t>1346146222</t>
-  </si>
-  <si>
-    <t>Flowmind LLC</t>
-  </si>
-  <si>
-    <t>Early Intervention Provider Agency</t>
-  </si>
-  <si>
-    <t>Middletown, DE</t>
-  </si>
-  <si>
-    <t>1114823341</t>
-  </si>
-  <si>
-    <t>Karie Swanner PMHNP-BC LLC</t>
-  </si>
-  <si>
-    <t>Nurse Practitioner</t>
-  </si>
-  <si>
-    <t>Milford, DE</t>
-  </si>
-  <si>
-    <t>1023914314</t>
-  </si>
-  <si>
-    <t>Virgo Integrated Health, LLC</t>
-  </si>
-  <si>
-    <t>Clinic/Center, Primary Care</t>
-  </si>
-  <si>
-    <t>Lewes, DE</t>
-  </si>
-  <si>
-    <t>1477459865</t>
-  </si>
-  <si>
-    <t>Delaware Psychotherapy</t>
-  </si>
-  <si>
-    <t>1073418844</t>
-  </si>
-  <si>
-    <t>Precious Care De LLC</t>
-  </si>
-  <si>
-    <t>Behavior Analyst</t>
-  </si>
-  <si>
-    <t>Rehoboth Beach, DE</t>
-  </si>
-  <si>
-    <t>1366347841</t>
-  </si>
-  <si>
-    <t>Align Speech LLC</t>
-  </si>
-  <si>
-    <t>Speech-Language Pathologist</t>
-  </si>
-  <si>
-    <t>Dagsboro, DE</t>
-  </si>
-  <si>
-    <t>1255236964</t>
-  </si>
-  <si>
-    <t>Diana Holness</t>
-  </si>
-  <si>
-    <t>Nurse Practitioner, Psychiatric/Mental Health</t>
-  </si>
-  <si>
-    <t>Felton, DE</t>
-  </si>
-  <si>
-    <t>1881599678</t>
-  </si>
-  <si>
-    <t>Chandler Fitzgerald</t>
-  </si>
-  <si>
-    <t>Social Worker, Clinical</t>
-  </si>
-  <si>
-    <t>Newark, DE</t>
-  </si>
-  <si>
-    <t>1811893761</t>
+    <t>Northland Adventure Education &amp; Therapy Center, Inc.</t>
+  </si>
+  <si>
+    <t>Addiction counselor</t>
+  </si>
+  <si>
+    <t>Moretown, VT</t>
+  </si>
+  <si>
+    <t>1285531285</t>
+  </si>
+  <si>
+    <t>The Kingdom Kares Maple Lane LLC</t>
+  </si>
+  <si>
+    <t>Skilled nursing facility</t>
+  </si>
+  <si>
+    <t>Barton, VT</t>
+  </si>
+  <si>
+    <t>1255237921</t>
+  </si>
+  <si>
+    <t>The Kingdom Kares Maple Lane Ops LLC</t>
+  </si>
+  <si>
+    <t>1952207623</t>
+  </si>
+  <si>
+    <t>The Kingdom Kares Pines Ops LLC</t>
+  </si>
+  <si>
+    <t>Lyndonville, VT</t>
+  </si>
+  <si>
+    <t>1669378345</t>
+  </si>
+  <si>
+    <t>The Kingdom Kares Union House Ops LLC</t>
+  </si>
+  <si>
+    <t>Glover, VT</t>
+  </si>
+  <si>
+    <t>1659277333</t>
+  </si>
+  <si>
+    <t>En Pointe Trauma Therapy &amp; Wellness PLC</t>
+  </si>
+  <si>
+    <t>Clinical social worker</t>
+  </si>
+  <si>
+    <t>Richmond, VT</t>
+  </si>
+  <si>
+    <t>1659278323</t>
+  </si>
+  <si>
+    <t>White Psychological Services, LLC</t>
+  </si>
+  <si>
+    <t>Psychologist</t>
+  </si>
+  <si>
+    <t>Barre, VT</t>
+  </si>
+  <si>
+    <t>1932006335</t>
+  </si>
+  <si>
+    <t>Firefly PLLC</t>
+  </si>
+  <si>
+    <t>Pediatric adolescent medicine physician</t>
+  </si>
+  <si>
+    <t>South Burlington, VT</t>
+  </si>
+  <si>
+    <t>1023914678</t>
+  </si>
+  <si>
+    <t>Little Rivers Health Care, Inc.</t>
+  </si>
+  <si>
+    <t>Pharmacist</t>
+  </si>
+  <si>
+    <t>Wells River, VT</t>
+  </si>
+  <si>
+    <t>1528964228</t>
+  </si>
+  <si>
+    <t>Rachel Jadkowski, PsyD, P.L.C.</t>
+  </si>
+  <si>
+    <t>Clinical psychologist</t>
+  </si>
+  <si>
+    <t>Richford, VT</t>
+  </si>
+  <si>
+    <t>1174429674</t>
   </si>
   <si>
     <t>How to work this list</t>
@@ -275,7 +269,7 @@
     <t>Every record comes from the public NPPES file published weekly by CMS (the federal NPI registry), as the provider filed it, and is provided as-is. Websites, emails and ratings are found on Google and the practice's own site. Click any NPI to see the official record.</t>
   </si>
   <si>
-    <t>New practices registered this week (Oct 12-Oct 18): Delaware</t>
+    <t>New practices registered this week (Oct 19-Oct 25): Vermont</t>
   </si>
   <si>
     <t>13 rows. Every new practice in your territory, sorted best-first with the top 25 highlighted. Click an NPI to open the official CMS record.</t>
@@ -332,346 +326,394 @@
     <t>Street address</t>
   </si>
   <si>
+    <t>Fax</t>
+  </si>
+  <si>
+    <t>License #</t>
+  </si>
+  <si>
+    <t>License state</t>
+  </si>
+  <si>
+    <t>Other specialties</t>
+  </si>
+  <si>
     <t>Taxonomy code</t>
   </si>
   <si>
     <t>Top 25</t>
   </si>
   <si>
-    <t>Maged Hosny</t>
-  </si>
-  <si>
-    <t>(302) 678-7438</t>
-  </si>
-  <si>
-    <t>Hi Maged, congratulations on registering Infusion Center of Delaware in Dover (Oct 15). New internal medicine, rheumatology practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+    <t>Edward Spaulding</t>
+  </si>
+  <si>
+    <t>Executive Director</t>
+  </si>
+  <si>
+    <t>(802) 858-4286</t>
+  </si>
+  <si>
+    <t>(802) 522-0675</t>
+  </si>
+  <si>
+    <t>Hi Edward, congratulations on registering Northland Adventure Education &amp; Therapy Center, Inc. in Moretown (Oct 22). New addiction counselor practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Behavioral Health</t>
+  </si>
+  <si>
+    <t>Moretown</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>05660</t>
+  </si>
+  <si>
+    <t>Hot: new organization; addiction counselor: heavy payer enrollment; name suggests a multi-provider practice; owner's own phone listed; registered in the last few days</t>
+  </si>
+  <si>
+    <t>Organization</t>
+  </si>
+  <si>
+    <t>31 Center Fayston Rd</t>
+  </si>
+  <si>
+    <t>(802) 329-2290</t>
+  </si>
+  <si>
+    <t>Counselor; Mental health counselor; Professional counselor; Addiction (substance use disorder) psychologist; Clinical psychologist; Exercise &amp; sports psychologist; Health service psychologist; Group psychotherapy psychologist; Social worker; Health educator; Health psychologist; Health &amp; wellness coach</t>
+  </si>
+  <si>
+    <t>101YA0400X</t>
+  </si>
+  <si>
+    <t>Travis Bergeron</t>
+  </si>
+  <si>
+    <t>Owner/CEO</t>
+  </si>
+  <si>
+    <t>(802) 745-7044</t>
+  </si>
+  <si>
+    <t>(802) 754-8575</t>
+  </si>
+  <si>
+    <t>Hi Travis, congratulations on registering The Kingdom Kares Maple Lane LLC in Barton (Oct 19). New skilled nursing facility practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Home Care &amp; Senior Living</t>
+  </si>
+  <si>
+    <t>Barton</t>
+  </si>
+  <si>
+    <t>05822</t>
+  </si>
+  <si>
+    <t>Hot: new organization; skilled nursing facility: heavy payer enrollment; owner's own phone listed</t>
+  </si>
+  <si>
+    <t>60 Maple Ln</t>
+  </si>
+  <si>
+    <t>314000000X</t>
+  </si>
+  <si>
+    <t>Hi Travis, congratulations on registering The Kingdom Kares Maple Lane Ops LLC in Barton (Oct 19). New skilled nursing facility practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>(802) 626-3361</t>
+  </si>
+  <si>
+    <t>Hi Travis, congratulations on registering The Kingdom Kares Pines Ops LLC in Lyndonville (Oct 19). New skilled nursing facility practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Lyndonville</t>
+  </si>
+  <si>
+    <t>05851</t>
+  </si>
+  <si>
+    <t>601 Red Village Rd</t>
+  </si>
+  <si>
+    <t>(802) 525-6600</t>
+  </si>
+  <si>
+    <t>Hi Travis, congratulations on registering The Kingdom Kares Union House Ops LLC in Glover (Oct 19). New skilled nursing facility practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Glover</t>
+  </si>
+  <si>
+    <t>05839</t>
+  </si>
+  <si>
+    <t>3086 Glover St</t>
+  </si>
+  <si>
+    <t>Amie Curran</t>
+  </si>
+  <si>
+    <t>Owner, Managing Member</t>
+  </si>
+  <si>
+    <t>(347) 619-7985</t>
+  </si>
+  <si>
+    <t>Hi Amie, congratulations on registering En Pointe Trauma Therapy &amp; Wellness PLC in Richmond (Oct 24). New clinical social worker practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Richmond</t>
+  </si>
+  <si>
+    <t>05477</t>
+  </si>
+  <si>
+    <t>Hot: new organization; clinical social worker: heavy payer enrollment; registered in the last few days</t>
+  </si>
+  <si>
+    <t>142 Church St</t>
+  </si>
+  <si>
+    <t>1041C0700X</t>
+  </si>
+  <si>
+    <t>Sarah White</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>(802) 522-4097</t>
+  </si>
+  <si>
+    <t>Hi Sarah, congratulations on registering White Psychological Services, LLC in Barre (Oct 20). New psychologist practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Barre</t>
+  </si>
+  <si>
+    <t>05641</t>
+  </si>
+  <si>
+    <t>Warm: new organization; psychologist; name suggests a multi-provider practice</t>
+  </si>
+  <si>
+    <t>14 N Main St Ste 1001</t>
+  </si>
+  <si>
+    <t>103T00000X</t>
+  </si>
+  <si>
+    <t>Erica Gibson</t>
+  </si>
+  <si>
+    <t>Director</t>
+  </si>
+  <si>
+    <t>(917) 488-9513</t>
+  </si>
+  <si>
+    <t>Hi Erica, congratulations on registering Firefly PLLC in South Burlington (Oct 19). New pediatric adolescent medicine physician practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
   </si>
   <si>
     <t>Medical Practices &amp; Clinics</t>
   </si>
   <si>
-    <t>Dover</t>
-  </si>
-  <si>
-    <t>DE</t>
-  </si>
-  <si>
-    <t>19904</t>
-  </si>
-  <si>
-    <t>Hot: new organization; internal medicine, rheumatology: heavy payer enrollment; name suggests a multi-provider practice; registered in the last few days</t>
-  </si>
-  <si>
-    <t>Organization</t>
-  </si>
-  <si>
-    <t>260 Beiser Blvd Ste 201</t>
-  </si>
-  <si>
-    <t>207RR0500X</t>
-  </si>
-  <si>
-    <t>Shree Shah</t>
-  </si>
-  <si>
-    <t>(415) 570-2350</t>
-  </si>
-  <si>
-    <t>Hi Shree, congratulations on registering Allminds Medical Group Midwest PA in Wilmington (Oct 16). New clinic/center, mental health (including community mental health center) practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>Behavioral Health</t>
-  </si>
-  <si>
-    <t>Wilmington</t>
-  </si>
-  <si>
-    <t>19801</t>
-  </si>
-  <si>
-    <t>Hot: new organization; clinic/center, mental health (including community mental health center): heavy payer enrollment; name suggests a multi-provider practice; registered in the last few days</t>
-  </si>
-  <si>
-    <t>1000 N West St Ste 1200</t>
-  </si>
-  <si>
-    <t>261QM0801X</t>
-  </si>
-  <si>
-    <t>Ni Dai</t>
-  </si>
-  <si>
-    <t>(347) 986-8678</t>
-  </si>
-  <si>
-    <t>Hi Ni, congratulations on registering Flowmind LLC in Middletown (Oct 15). New early intervention provider agency practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>Home Care &amp; Senior Living</t>
-  </si>
-  <si>
-    <t>Middletown</t>
-  </si>
-  <si>
-    <t>19709</t>
-  </si>
-  <si>
-    <t>Warm: new organization; early intervention provider agency; registered in the last few days</t>
-  </si>
-  <si>
-    <t>300 Jessica Dr</t>
-  </si>
-  <si>
-    <t>252Y00000X</t>
-  </si>
-  <si>
-    <t>Karie Swanner</t>
-  </si>
-  <si>
-    <t>(443) 871-1247</t>
-  </si>
-  <si>
-    <t>Hi Karie, congratulations on registering Karie Swanner Pmhnp-Bc LLC in Milford (Oct 15). New nurse practitioner practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>Milford</t>
-  </si>
-  <si>
-    <t>19963</t>
-  </si>
-  <si>
-    <t>Warm: new organization; nurse practitioner: heavy payer enrollment; looks like a one-person PLLC; registered in the last few days</t>
-  </si>
-  <si>
-    <t>18 SW Front St Unit 111</t>
-  </si>
-  <si>
-    <t>363L00000X</t>
-  </si>
-  <si>
-    <t>Danielle Giddins</t>
-  </si>
-  <si>
-    <t>(302) 313-1964</t>
-  </si>
-  <si>
-    <t>Hi Danielle, congratulations on registering Virgo Integrated Health, LLC in Lewes (Oct 14). New clinic/center, primary care practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>Lewes</t>
-  </si>
-  <si>
-    <t>19958</t>
-  </si>
-  <si>
-    <t>Warm: new organization; clinic/center, primary care: heavy payer enrollment</t>
-  </si>
-  <si>
-    <t>1632 Savannah Rd</t>
-  </si>
-  <si>
-    <t>261QP2300X</t>
-  </si>
-  <si>
-    <t>Elizabeth Brown</t>
-  </si>
-  <si>
-    <t>(540) 974-4308</t>
-  </si>
-  <si>
-    <t>Hi Elizabeth, congratulations on registering Delaware Psychotherapy in Wilmington (Oct 12). New clinic/center, mental health (including community mental health center) practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>19806</t>
-  </si>
-  <si>
-    <t>Warm: new organization; clinic/center, mental health (including community mental health center): heavy payer enrollment</t>
-  </si>
-  <si>
-    <t>1803 Shallcross Ave</t>
-  </si>
-  <si>
-    <t>Rochelle Zwick</t>
-  </si>
-  <si>
-    <t>(888) 815-9287</t>
-  </si>
-  <si>
-    <t>Hi Rochelle, congratulations on registering Precious Care De LLC in Rehoboth Beach (Oct 13). New behavior analyst practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>Rehoboth Beach</t>
-  </si>
-  <si>
-    <t>19971</t>
-  </si>
-  <si>
-    <t>Warm: new organization; behavior analyst: heavy payer enrollment</t>
-  </si>
-  <si>
-    <t>511 N Boardwalk</t>
-  </si>
-  <si>
-    <t>103K00000X</t>
-  </si>
-  <si>
-    <t>Shannon Yacucci</t>
-  </si>
-  <si>
-    <t>(302) 757-6537</t>
-  </si>
-  <si>
-    <t>Hi Shannon, congratulations on registering Align Speech LLC in Dagsboro (Oct 12). New speech-language pathologist practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
-  </si>
-  <si>
-    <t>Therapy &amp; Rehab</t>
-  </si>
-  <si>
-    <t>Dagsboro</t>
-  </si>
-  <si>
-    <t>19939</t>
-  </si>
-  <si>
-    <t>Warm: new organization; speech-language pathologist: heavy payer enrollment</t>
-  </si>
-  <si>
-    <t>31186 Dogwood Acres Rd</t>
-  </si>
-  <si>
-    <t>235Z00000X</t>
-  </si>
-  <si>
-    <t>(862) 252-3517</t>
-  </si>
-  <si>
-    <t>Hi Diana, congratulations on starting your own nurse practitioner, psychiatric/mental health practice in Felton (Oct 12). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
-  </si>
-  <si>
-    <t>Felton</t>
-  </si>
-  <si>
-    <t>19943</t>
-  </si>
-  <si>
-    <t>Cool: sole proprietor; nurse practitioner, psychiatric/mental health: heavy payer enrollment</t>
+    <t>South Burlington</t>
+  </si>
+  <si>
+    <t>05403</t>
+  </si>
+  <si>
+    <t>Warm: new organization; pediatric adolescent medicine physician</t>
+  </si>
+  <si>
+    <t>65 Central Ave</t>
+  </si>
+  <si>
+    <t>2080A0000X</t>
+  </si>
+  <si>
+    <t>Andrew Barter</t>
+  </si>
+  <si>
+    <t>CEO</t>
+  </si>
+  <si>
+    <t>(802) 222-3023</t>
+  </si>
+  <si>
+    <t>(802) 222-3090</t>
+  </si>
+  <si>
+    <t>Hi Andrew, congratulations on registering Little Rivers Health Care, Inc. in Wells River (Oct 19). New pharmacist practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>DME, Pharmacy &amp; Transport</t>
+  </si>
+  <si>
+    <t>Wells River</t>
+  </si>
+  <si>
+    <t>05081</t>
+  </si>
+  <si>
+    <t>Warm: new organization; pharmacist: rarely outsources credentialing; name suggests a multi-provider practice; owner's own phone listed</t>
+  </si>
+  <si>
+    <t>55 Main St N</t>
+  </si>
+  <si>
+    <t>(855) 868-7197</t>
+  </si>
+  <si>
+    <t>Dentist, general; Dental hygienist; Pharmacy technician; Family medicine</t>
+  </si>
+  <si>
+    <t>183500000X</t>
+  </si>
+  <si>
+    <t>Rachel Jadkowski</t>
+  </si>
+  <si>
+    <t>(802) 441-7105</t>
+  </si>
+  <si>
+    <t>Hi Rachel, congratulations on registering Rachel Jadkowski, PSYD, P.L.C. in Richford (Oct 20). New clinical psychologist practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Richford</t>
+  </si>
+  <si>
+    <t>05476</t>
+  </si>
+  <si>
+    <t>Warm: new organization; clinical psychologist; looks like a one-person PLLC</t>
+  </si>
+  <si>
+    <t>40 Green Mountain Rd</t>
+  </si>
+  <si>
+    <t>103TC0700X</t>
+  </si>
+  <si>
+    <t>Danielle Witte</t>
+  </si>
+  <si>
+    <t>(352) 857-7613</t>
+  </si>
+  <si>
+    <t>Hi Danielle, congratulations on starting your own mental health counselor practice in North Troy (Oct 23). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
+  </si>
+  <si>
+    <t>Mental health counselor</t>
+  </si>
+  <si>
+    <t>North Troy</t>
+  </si>
+  <si>
+    <t>05859</t>
+  </si>
+  <si>
+    <t>Cool: sole proprietor; mental health counselor: heavy payer enrollment; registered in the last few days</t>
   </si>
   <si>
     <t>Solo provider</t>
   </si>
   <si>
-    <t>PMHNP</t>
-  </si>
-  <si>
-    <t>349 Belfry Dr</t>
-  </si>
-  <si>
-    <t>363LP0808X</t>
-  </si>
-  <si>
-    <t>(302) 312-4217</t>
-  </si>
-  <si>
-    <t>Hi Chandler, congratulations on starting your own social worker, clinical practice in Newark (Oct 16). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
-  </si>
-  <si>
-    <t>Newark</t>
-  </si>
-  <si>
-    <t>19713</t>
-  </si>
-  <si>
-    <t>Cool: sole proprietor; social worker, clinical: heavy payer enrollment; LMSW credential (often not billing independently yet); registered in the last few days</t>
-  </si>
-  <si>
-    <t>LMSW</t>
-  </si>
-  <si>
-    <t>100 Commerce Dr</t>
-  </si>
-  <si>
-    <t>1041C0700X</t>
-  </si>
-  <si>
-    <t>Christina Hernandez</t>
-  </si>
-  <si>
-    <t>(857) 557-6146</t>
-  </si>
-  <si>
-    <t>Hi Christina, congratulations on starting your own social worker practice in Lewes (Oct 13). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
-  </si>
-  <si>
-    <t>Social Worker</t>
-  </si>
-  <si>
-    <t>Cool: sole proprietor; social worker</t>
-  </si>
-  <si>
-    <t>16192 Coastal Hwy</t>
-  </si>
-  <si>
-    <t>1235034737</t>
-  </si>
-  <si>
-    <t>104100000X</t>
-  </si>
-  <si>
-    <t>Yaw Asante</t>
-  </si>
-  <si>
-    <t>(302) 390-2266</t>
-  </si>
-  <si>
-    <t>Hi Yaw, congratulations on starting your own behavior technician practice in Townsend (Oct 13). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
-  </si>
-  <si>
-    <t>Behavior Technician</t>
-  </si>
-  <si>
-    <t>Townsend</t>
-  </si>
-  <si>
-    <t>19734</t>
-  </si>
-  <si>
-    <t>Cool: sole proprietor; behavior technician</t>
-  </si>
-  <si>
-    <t>146 Abbigail Xing</t>
-  </si>
-  <si>
-    <t>1518862028</t>
-  </si>
-  <si>
-    <t>106S00000X</t>
-  </si>
-  <si>
-    <t>Hassan Kaleem</t>
-  </si>
-  <si>
-    <t>(302) 747-5995</t>
-  </si>
-  <si>
-    <t>Hi Dr. Kaleem, congratulations on starting your own physical therapist, orthopedic practice in Dover (Oct 12). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
-  </si>
-  <si>
-    <t>Physical Therapist, Orthopedic</t>
-  </si>
-  <si>
-    <t>Cool: sole proprietor</t>
-  </si>
-  <si>
-    <t>DPT</t>
-  </si>
-  <si>
-    <t>285 Beiser Blvd</t>
-  </si>
-  <si>
-    <t>1982509733</t>
-  </si>
-  <si>
-    <t>2251X0800X</t>
+    <t>CMHC</t>
+  </si>
+  <si>
+    <t>80 School St</t>
+  </si>
+  <si>
+    <t>068.0137518</t>
+  </si>
+  <si>
+    <t>1760389621</t>
+  </si>
+  <si>
+    <t>101YM0800X</t>
+  </si>
+  <si>
+    <t>Lume Business LLC</t>
+  </si>
+  <si>
+    <t>Kleber Cortes Bonifacio</t>
+  </si>
+  <si>
+    <t>(407) 842-9152</t>
+  </si>
+  <si>
+    <t>Hi Kleber, congratulations on registering Lume Business LLC in Williston (Oct 20). New dentist practices usually start payer credentialing in the first 60-90 days: are you handling that in-house, or would help be useful?</t>
+  </si>
+  <si>
+    <t>Dentist</t>
+  </si>
+  <si>
+    <t>Dental</t>
+  </si>
+  <si>
+    <t>Williston</t>
+  </si>
+  <si>
+    <t>05495</t>
+  </si>
+  <si>
+    <t>Cool: new organization; dentist: rarely outsources credentialing</t>
+  </si>
+  <si>
+    <t>75 Talcott Rd Ste 60</t>
+  </si>
+  <si>
+    <t>Dental hygienist</t>
+  </si>
+  <si>
+    <t>1265338768</t>
+  </si>
+  <si>
+    <t>122300000X</t>
+  </si>
+  <si>
+    <t>Stephanie Wales</t>
+  </si>
+  <si>
+    <t>(603) 387-5633</t>
+  </si>
+  <si>
+    <t>Hi Stephanie, congratulations on starting your own school psychologist practice in East Haven (Oct 20). Have you started getting credentialed with insurance plans yet, or is that still on the to-do list?</t>
+  </si>
+  <si>
+    <t>School psychologist</t>
+  </si>
+  <si>
+    <t>East Haven</t>
+  </si>
+  <si>
+    <t>05837</t>
+  </si>
+  <si>
+    <t>Cool: sole proprietor; school psychologist</t>
+  </si>
+  <si>
+    <t>1881 Vt Route 114</t>
+  </si>
+  <si>
+    <t>77640</t>
+  </si>
+  <si>
+    <t>NH</t>
+  </si>
+  <si>
+    <t>1952208464</t>
+  </si>
+  <si>
+    <t>103TS0200X</t>
   </si>
   <si>
     <t>How to use your list</t>
@@ -1734,7 +1776,7 @@
     </row>
     <row r="16" spans="2:9" ht="18" customHeight="1">
       <c r="B16" s="12">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>14</v>
@@ -1754,7 +1796,7 @@
     </row>
     <row r="17" spans="2:9" ht="18" customHeight="1">
       <c r="B17" s="12">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>18</v>
@@ -1774,7 +1816,7 @@
     </row>
     <row r="18" spans="2:9" ht="18" customHeight="1">
       <c r="B18" s="12">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>22</v>
@@ -1782,74 +1824,74 @@
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G18" s="13"/>
       <c r="H18" s="13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="18" customHeight="1">
       <c r="B19" s="12">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="13" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G19" s="13"/>
       <c r="H19" s="13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="18" customHeight="1">
       <c r="B20" s="12">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="13" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G20" s="13"/>
       <c r="H20" s="13" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="18" customHeight="1">
       <c r="B21" s="12">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="13"/>
       <c r="F21" s="13" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="G21" s="13"/>
       <c r="H21" s="13" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="18" customHeight="1">
@@ -1857,84 +1899,84 @@
         <v>77</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G22" s="13"/>
       <c r="H22" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23" spans="2:9" ht="18" customHeight="1">
       <c r="B23" s="12">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G23" s="13"/>
       <c r="H23" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="2:9" ht="18" customHeight="1">
       <c r="B24" s="12">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
       <c r="F24" s="13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G24" s="13"/>
       <c r="H24" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="2:9" ht="18" customHeight="1">
       <c r="B25" s="12">
+        <v>65</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>46</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>48</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="13"/>
       <c r="F25" s="13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G25" s="13"/>
       <c r="H25" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="21.75" customHeight="1">
       <c r="B27" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="2:9" ht="36" customHeight="1">
@@ -1942,7 +1984,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
@@ -1956,7 +1998,7 @@
         <v>2</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
@@ -1970,7 +2012,7 @@
         <v>3</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
@@ -1981,16 +2023,16 @@
     </row>
     <row r="32" spans="2:9" ht="21.75" customHeight="1">
       <c r="B32" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="33.75" customHeight="1">
       <c r="B33" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C33" s="16"/>
       <c r="D33" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
@@ -2000,11 +2042,11 @@
     </row>
     <row r="34" spans="2:9" ht="18.75" customHeight="1">
       <c r="B34" s="16" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C34" s="16"/>
       <c r="D34" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
@@ -2014,11 +2056,11 @@
     </row>
     <row r="36" spans="2:9" ht="27.75" customHeight="1">
       <c r="B36" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C36" s="17"/>
       <c r="D36" s="18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E36" s="18"/>
       <c r="F36" s="18"/>
@@ -2028,7 +2070,7 @@
     </row>
     <row r="38" spans="2:9" ht="18" customHeight="1">
       <c r="B38" s="19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C38" s="19"/>
       <c r="D38" s="19"/>
@@ -2122,7 +2164,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -2144,879 +2186,995 @@
     <col min="18" max="18" width="13.7109375" customWidth="1"/>
     <col min="19" max="19" width="11.7109375" customWidth="1"/>
     <col min="20" max="20" width="30.7109375" customWidth="1"/>
-    <col min="21" max="21" width="12.7109375" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
     <col min="22" max="22" width="13.7109375" customWidth="1"/>
+    <col min="23" max="23" width="8.7109375" customWidth="1"/>
+    <col min="24" max="24" width="30.7109375" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
+    <col min="26" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="36" customHeight="1">
+    <row r="1" spans="1:26" ht="36" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="21.75" customHeight="1">
+    <row r="2" spans="1:26" ht="21.75" customHeight="1">
       <c r="A2" s="20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="17.25" customHeight="1">
+      <c r="A3" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="30" customHeight="1">
+      <c r="A4" s="22" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:22" ht="17.25" customHeight="1">
-      <c r="A3" s="21" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" ht="30" customHeight="1">
-      <c r="A4" s="22" t="s">
-        <v>66</v>
       </c>
       <c r="B4" s="22" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="E4" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="F4" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="G4" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="H4" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="I4" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="J4" s="22" t="s">
         <v>72</v>
-      </c>
-      <c r="I4" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="J4" s="22" t="s">
-        <v>74</v>
       </c>
       <c r="K4" s="22" t="s">
         <v>11</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M4" s="22" t="s">
         <v>12</v>
       </c>
       <c r="N4" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="O4" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="P4" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="O4" s="22" t="s">
+      <c r="Q4" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="P4" s="22" t="s">
+      <c r="R4" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="Q4" s="22" t="s">
+      <c r="S4" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="R4" s="22" t="s">
+      <c r="T4" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="S4" s="22" t="s">
+      <c r="U4" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="T4" s="22" t="s">
+      <c r="V4" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="U4" s="22" t="s">
+      <c r="W4" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="X4" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="Y4" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="V4" s="22" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22">
+      <c r="Z4" s="22" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26">
       <c r="A5" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B5" s="24">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C5" s="25" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
+        <v>87</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>89</v>
+      </c>
       <c r="G5" s="25" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H5" s="25"/>
       <c r="I5" s="25"/>
       <c r="J5" s="25" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="K5" s="25" t="s">
         <v>15</v>
       </c>
       <c r="L5" s="25" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="M5" s="25" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="N5" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O5" s="25" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="P5" s="26">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="Q5" s="25" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="R5" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S5" s="25"/>
       <c r="T5" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="U5" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="U5" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="V5" s="25"/>
+      <c r="W5" s="25"/>
+      <c r="X5" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y5" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="V5" s="25" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22">
+      <c r="Z5" s="25" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26">
       <c r="A6" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="24">
         <v>84</v>
-      </c>
-      <c r="B6" s="24">
-        <v>89</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
+        <v>102</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>104</v>
+      </c>
       <c r="G6" s="25" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H6" s="25"/>
       <c r="I6" s="25"/>
       <c r="J6" s="25" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="K6" s="25" t="s">
         <v>19</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="N6" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O6" s="25" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="P6" s="26">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="R6" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S6" s="25"/>
       <c r="T6" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="U6" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="U6" s="25"/>
+      <c r="V6" s="25"/>
+      <c r="W6" s="25"/>
+      <c r="X6" s="25"/>
+      <c r="Y6" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="V6" s="25" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22">
+      <c r="Z6" s="25" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26">
       <c r="A7" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="24">
         <v>84</v>
-      </c>
-      <c r="B7" s="24">
-        <v>78</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="G7" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="H7" s="25"/>
       <c r="I7" s="25"/>
       <c r="J7" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="K7" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="L7" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="K7" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="L7" s="25" t="s">
+      <c r="M7" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="M7" s="25" t="s">
+      <c r="N7" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="O7" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="N7" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="O7" s="25" t="s">
+      <c r="P7" s="26">
+        <v>46314</v>
+      </c>
+      <c r="Q7" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="P7" s="26">
-        <v>46310</v>
-      </c>
-      <c r="Q7" s="25" t="s">
-        <v>111</v>
-      </c>
       <c r="R7" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S7" s="25"/>
       <c r="T7" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="U7" s="25"/>
+      <c r="V7" s="25"/>
+      <c r="W7" s="25"/>
+      <c r="X7" s="25"/>
+      <c r="Y7" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z7" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="U7" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="V7" s="25" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22">
+    </row>
+    <row r="8" spans="1:26">
       <c r="A8" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="24">
         <v>84</v>
       </c>
-      <c r="B8" s="24">
-        <v>78</v>
-      </c>
       <c r="C8" s="25" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" s="25" t="s">
         <v>114</v>
-      </c>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25" t="s">
-        <v>115</v>
       </c>
       <c r="H8" s="25"/>
       <c r="I8" s="25"/>
       <c r="J8" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="K8" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="L8" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="M8" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="K8" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="M8" s="25" t="s">
+      <c r="N8" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="O8" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="N8" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="O8" s="25" t="s">
-        <v>118</v>
-      </c>
       <c r="P8" s="26">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="Q8" s="25" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="R8" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S8" s="25"/>
       <c r="T8" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="U8" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="V8" s="25" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22">
+        <v>118</v>
+      </c>
+      <c r="U8" s="25"/>
+      <c r="V8" s="25"/>
+      <c r="W8" s="25"/>
+      <c r="X8" s="25"/>
+      <c r="Y8" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z8" s="25" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26">
       <c r="A9" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="24">
         <v>84</v>
       </c>
-      <c r="B9" s="24">
-        <v>78</v>
-      </c>
       <c r="C9" s="25" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
+        <v>102</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>104</v>
+      </c>
       <c r="G9" s="25" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H9" s="25"/>
       <c r="I9" s="25"/>
       <c r="J9" s="25" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="K9" s="25" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="L9" s="25" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="M9" s="25" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="N9" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O9" s="25" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="P9" s="26">
-        <v>46309</v>
+        <v>46314</v>
       </c>
       <c r="Q9" s="25" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="R9" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S9" s="25"/>
       <c r="T9" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="U9" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="V9" s="25" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22">
+        <v>123</v>
+      </c>
+      <c r="U9" s="25"/>
+      <c r="V9" s="25"/>
+      <c r="W9" s="25"/>
+      <c r="X9" s="25"/>
+      <c r="Y9" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z9" s="25" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26">
       <c r="A10" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B10" s="24">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="E10" s="25"/>
+        <v>124</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>125</v>
+      </c>
       <c r="F10" s="25"/>
       <c r="G10" s="25" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="H10" s="25"/>
       <c r="I10" s="25"/>
       <c r="J10" s="25" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K10" s="25" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="L10" s="25" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M10" s="25" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
       <c r="N10" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O10" s="25" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="P10" s="26">
-        <v>46307</v>
+        <v>46319</v>
       </c>
       <c r="Q10" s="25" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="R10" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S10" s="25"/>
       <c r="T10" s="25" t="s">
-        <v>135</v>
-      </c>
-      <c r="U10" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="V10" s="25" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22">
+        <v>131</v>
+      </c>
+      <c r="U10" s="25"/>
+      <c r="V10" s="25"/>
+      <c r="W10" s="25"/>
+      <c r="X10" s="25"/>
+      <c r="Y10" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z10" s="25" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26">
       <c r="A11" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B11" s="24">
         <v>77</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>136</v>
-      </c>
-      <c r="E11" s="25"/>
+        <v>133</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>134</v>
+      </c>
       <c r="F11" s="25"/>
       <c r="G11" s="25" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H11" s="25"/>
       <c r="I11" s="25"/>
       <c r="J11" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="K11" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="L11" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="M11" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="N11" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="O11" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="K11" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="L11" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="M11" s="25" t="s">
+      <c r="P11" s="26">
+        <v>46315</v>
+      </c>
+      <c r="Q11" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="N11" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="O11" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="P11" s="26">
-        <v>46308</v>
-      </c>
-      <c r="Q11" s="25" t="s">
-        <v>141</v>
-      </c>
       <c r="R11" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S11" s="25"/>
       <c r="T11" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="U11" s="25"/>
+      <c r="V11" s="25"/>
+      <c r="W11" s="25"/>
+      <c r="X11" s="25"/>
+      <c r="Y11" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z11" s="25" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="24">
+        <v>70</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="U11" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="V11" s="25" t="s">
+      <c r="E12" s="25" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="12" spans="1:22">
-      <c r="A12" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="B12" s="24">
-        <v>72</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="E12" s="25"/>
       <c r="F12" s="25"/>
       <c r="G12" s="25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H12" s="25"/>
       <c r="I12" s="25"/>
       <c r="J12" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="K12" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="L12" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="K12" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="L12" s="25" t="s">
+      <c r="M12" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="M12" s="25" t="s">
+      <c r="N12" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="O12" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="N12" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="O12" s="25" t="s">
+      <c r="P12" s="26">
+        <v>46314</v>
+      </c>
+      <c r="Q12" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="P12" s="26">
-        <v>46307</v>
-      </c>
-      <c r="Q12" s="25" t="s">
-        <v>150</v>
-      </c>
       <c r="R12" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="S12" s="25"/>
       <c r="T12" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="U12" s="25"/>
+      <c r="V12" s="25"/>
+      <c r="W12" s="25"/>
+      <c r="X12" s="25"/>
+      <c r="Y12" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z12" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="U12" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="V12" s="25" t="s">
+    </row>
+    <row r="13" spans="1:26">
+      <c r="A13" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="24">
+        <v>70</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="25" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="13" spans="1:22">
-      <c r="A13" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="B13" s="24">
-        <v>52</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
+      <c r="E13" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>154</v>
+      </c>
       <c r="G13" s="25" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H13" s="25"/>
       <c r="I13" s="25"/>
       <c r="J13" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K13" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="L13" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="M13" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="N13" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="O13" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="P13" s="26">
+        <v>46314</v>
+      </c>
+      <c r="Q13" s="25" t="s">
+        <v>160</v>
+      </c>
+      <c r="R13" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="S13" s="25"/>
+      <c r="T13" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="U13" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="V13" s="25"/>
+      <c r="W13" s="25"/>
+      <c r="X13" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y13" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="L13" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="M13" s="25" t="s">
-        <v>155</v>
-      </c>
-      <c r="N13" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="O13" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="P13" s="26">
-        <v>46307</v>
-      </c>
-      <c r="Q13" s="25" t="s">
-        <v>157</v>
-      </c>
-      <c r="R13" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="S13" s="25" t="s">
-        <v>159</v>
-      </c>
-      <c r="T13" s="25" t="s">
-        <v>160</v>
-      </c>
-      <c r="U13" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="V13" s="25" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22">
+      <c r="Z13" s="25" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26">
       <c r="A14" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B14" s="24">
+        <v>65</v>
+      </c>
+      <c r="C14" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="25" t="s">
-        <v>48</v>
-      </c>
       <c r="D14" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="25"/>
+        <v>165</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>134</v>
+      </c>
       <c r="F14" s="25"/>
       <c r="G14" s="25" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="H14" s="25"/>
       <c r="I14" s="25"/>
       <c r="J14" s="25" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="K14" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="L14" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="M14" s="25" t="s">
+        <v>168</v>
+      </c>
+      <c r="N14" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="O14" s="25" t="s">
+        <v>169</v>
+      </c>
+      <c r="P14" s="26">
+        <v>46315</v>
+      </c>
+      <c r="Q14" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="R14" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="S14" s="25"/>
+      <c r="T14" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="U14" s="25"/>
+      <c r="V14" s="25"/>
+      <c r="W14" s="25"/>
+      <c r="X14" s="25"/>
+      <c r="Y14" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="L14" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="M14" s="25" t="s">
-        <v>164</v>
-      </c>
-      <c r="N14" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="O14" s="25" t="s">
-        <v>165</v>
-      </c>
-      <c r="P14" s="26">
-        <v>46311</v>
-      </c>
-      <c r="Q14" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="R14" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="S14" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="T14" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="U14" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="V14" s="25" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22">
+      <c r="Z14" s="25" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26">
       <c r="A15" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B15" s="24">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E15" s="25"/>
       <c r="F15" s="25"/>
       <c r="G15" s="25" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H15" s="25"/>
       <c r="I15" s="25"/>
       <c r="J15" s="25" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="K15" s="25" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="L15" s="25" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M15" s="25" t="s">
-        <v>125</v>
+        <v>177</v>
       </c>
       <c r="N15" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O15" s="25" t="s">
-        <v>126</v>
+        <v>178</v>
       </c>
       <c r="P15" s="26">
-        <v>46308</v>
+        <v>46318</v>
       </c>
       <c r="Q15" s="25" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="R15" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="S15" s="25"/>
+        <v>180</v>
+      </c>
+      <c r="S15" s="25" t="s">
+        <v>181</v>
+      </c>
       <c r="T15" s="25" t="s">
-        <v>175</v>
-      </c>
-      <c r="U15" s="27" t="s">
-        <v>176</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="U15" s="25"/>
       <c r="V15" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22">
+        <v>183</v>
+      </c>
+      <c r="W15" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="X15" s="25"/>
+      <c r="Y15" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z15" s="25" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26">
       <c r="A16" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B16" s="24">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>178</v>
-      </c>
-      <c r="E16" s="25"/>
+        <v>187</v>
+      </c>
+      <c r="E16" s="25" t="s">
+        <v>134</v>
+      </c>
       <c r="F16" s="25"/>
       <c r="G16" s="25" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="H16" s="25"/>
       <c r="I16" s="25"/>
       <c r="J16" s="25" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="K16" s="25" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="L16" s="25" t="s">
-        <v>99</v>
+        <v>191</v>
       </c>
       <c r="M16" s="25" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="N16" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O16" s="25" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="P16" s="26">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="Q16" s="25" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="R16" s="25" t="s">
-        <v>158</v>
+        <v>97</v>
       </c>
       <c r="S16" s="25"/>
       <c r="T16" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="U16" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="V16" s="25" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="17" spans="1:22">
+        <v>195</v>
+      </c>
+      <c r="U16" s="25"/>
+      <c r="V16" s="25"/>
+      <c r="W16" s="25"/>
+      <c r="X16" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="Y16" s="27" t="s">
+        <v>197</v>
+      </c>
+      <c r="Z16" s="25" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26">
       <c r="A17" s="23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B17" s="24">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="E17" s="25"/>
       <c r="F17" s="25"/>
       <c r="G17" s="25" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="H17" s="25"/>
       <c r="I17" s="25"/>
       <c r="J17" s="25" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="K17" s="25" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="L17" s="25" t="s">
-        <v>147</v>
+        <v>92</v>
       </c>
       <c r="M17" s="25" t="s">
-        <v>89</v>
+        <v>203</v>
       </c>
       <c r="N17" s="25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="O17" s="25" t="s">
-        <v>91</v>
+        <v>204</v>
       </c>
       <c r="P17" s="26">
-        <v>46307</v>
+        <v>46315</v>
       </c>
       <c r="Q17" s="25" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="R17" s="25" t="s">
-        <v>158</v>
-      </c>
-      <c r="S17" s="25" t="s">
-        <v>193</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="S17" s="25"/>
       <c r="T17" s="25" t="s">
-        <v>194</v>
-      </c>
-      <c r="U17" s="27" t="s">
-        <v>195</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="U17" s="25"/>
       <c r="V17" s="25" t="s">
-        <v>196</v>
+        <v>207</v>
+      </c>
+      <c r="W17" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="X17" s="25"/>
+      <c r="Y17" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="Z17" s="25" t="s">
+        <v>210</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:V17"/>
+  <autoFilter ref="A4:Z17"/>
   <conditionalFormatting sqref="A5:A17">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Top 25"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:V17">
+  <conditionalFormatting sqref="A5:Z17">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="U5" r:id="rId1"/>
-    <hyperlink ref="U6" r:id="rId2"/>
-    <hyperlink ref="U7" r:id="rId3"/>
-    <hyperlink ref="U8" r:id="rId4"/>
-    <hyperlink ref="U9" r:id="rId5"/>
-    <hyperlink ref="U10" r:id="rId6"/>
-    <hyperlink ref="U11" r:id="rId7"/>
-    <hyperlink ref="U12" r:id="rId8"/>
-    <hyperlink ref="U13" r:id="rId9"/>
-    <hyperlink ref="U14" r:id="rId10"/>
-    <hyperlink ref="U15" r:id="rId11"/>
-    <hyperlink ref="U16" r:id="rId12"/>
-    <hyperlink ref="U17" r:id="rId13"/>
+    <hyperlink ref="Y5" r:id="rId1"/>
+    <hyperlink ref="Y6" r:id="rId2"/>
+    <hyperlink ref="Y7" r:id="rId3"/>
+    <hyperlink ref="Y8" r:id="rId4"/>
+    <hyperlink ref="Y9" r:id="rId5"/>
+    <hyperlink ref="Y10" r:id="rId6"/>
+    <hyperlink ref="Y11" r:id="rId7"/>
+    <hyperlink ref="Y12" r:id="rId8"/>
+    <hyperlink ref="Y13" r:id="rId9"/>
+    <hyperlink ref="Y14" r:id="rId10"/>
+    <hyperlink ref="Y15" r:id="rId11"/>
+    <hyperlink ref="Y16" r:id="rId12"/>
+    <hyperlink ref="Y17" r:id="rId13"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.7" bottom="0.6" header="0.3" footer="0.3"/>
@@ -3026,7 +3184,7 @@
     <oddFooter>&amp;L&amp;8&amp;K5B6B82PanelReady  ·  public data from the CMS NPI registry&amp;R&amp;8&amp;K5B6B82Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="A1:V17" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:Z17" numberStoredAsText="1"/>
   </ignoredErrors>
   <drawing r:id="rId14"/>
   <legacyDrawingHF r:id="rId15"/>
@@ -3055,181 +3213,181 @@
     </row>
     <row r="4" spans="2:3" ht="30" customHeight="1">
       <c r="B4" s="4" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="21.75" customHeight="1">
       <c r="B6" s="10" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="33.75" customHeight="1">
       <c r="B7" s="28" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="33.75" customHeight="1">
       <c r="B8" s="28" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="33.75" customHeight="1">
       <c r="B9" s="28" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="21.75" customHeight="1">
       <c r="B11" s="10" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="62.25" customHeight="1">
       <c r="B12" s="29" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="C12" s="29"/>
     </row>
     <row r="13" spans="2:3">
       <c r="B13" s="6" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="C13" s="6"/>
     </row>
     <row r="15" spans="2:3" ht="21.75" customHeight="1">
       <c r="B15" s="10" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="120" customHeight="1">
       <c r="B16" s="30" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="C16" s="30"/>
     </row>
     <row r="18" spans="2:3" ht="21.75" customHeight="1">
       <c r="B18" s="10" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="33.75" customHeight="1">
       <c r="B19" s="31" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="33.75" customHeight="1">
       <c r="B20" s="31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C20" s="32" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="19.5" customHeight="1">
       <c r="B21" s="31" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="C21" s="32" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="33.75" customHeight="1">
       <c r="B22" s="31" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C22" s="32" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="33.75" customHeight="1">
       <c r="B23" s="31" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="C23" s="32" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="33.75" customHeight="1">
       <c r="B24" s="31" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C24" s="32" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="19.5" customHeight="1">
       <c r="B25" s="31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C25" s="32" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="48.75" customHeight="1">
       <c r="B26" s="31" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="C26" s="32" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="19.5" customHeight="1">
       <c r="B27" s="31" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="C27" s="32" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="33.75" customHeight="1">
       <c r="B28" s="31" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="C28" s="32" t="s">
-        <v>227</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="33.75" customHeight="1">
       <c r="B29" s="31" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="C29" s="32" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="19.5" customHeight="1">
       <c r="B30" s="31" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="C30" s="32" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="33.75" customHeight="1">
       <c r="B31" s="31" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="C31" s="32" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="33.75" customHeight="1">
       <c r="B32" s="31" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="C32" s="32" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="19.5" customHeight="1">
@@ -3237,50 +3395,50 @@
         <v>13</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="2:3" ht="19.5" customHeight="1">
       <c r="B34" s="31" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="C34" s="32" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" spans="2:3" ht="19.5" customHeight="1">
       <c r="B35" s="31" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="C35" s="32" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="33.75" customHeight="1">
       <c r="B36" s="31" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="C36" s="32" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
     </row>
     <row r="37" spans="2:3" ht="33.75" customHeight="1">
       <c r="B37" s="31" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="C37" s="32" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39" spans="2:3" ht="30" customHeight="1">
       <c r="B39" s="28" t="s">
-        <v>245</v>
+        <v>259</v>
       </c>
       <c r="C39" s="28"/>
     </row>
     <row r="41" spans="2:3">
       <c r="B41" s="19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C41" s="19"/>
     </row>

</xml_diff>